<commit_message>
Add cards-resource, hero-gradient blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/cards-resource/cards-resource.css
- blocks/hero-gradient/hero-gradient.css
- blocks/hero-gradient/hero-gradient.js
- tools/importer/import-homepage.bundle.js
- tools/importer/parsers/hero-gradient.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -55,7 +55,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-03-30T19:06:33.010Z</t>
+    <t>2026-03-31T02:19:03.586Z</t>
   </si>
   <si>
     <t>Ancestry - Family Tree, Genealogy &amp; Family History Records</t>
@@ -76,7 +76,7 @@
     <t>product-landing</t>
   </si>
   <si>
-    <t>2026-03-30T18:47:28.966Z</t>
+    <t>2026-03-30T19:06:53.867Z</t>
   </si>
   <si>
     <t>Family History | Ancestry</t>
@@ -97,7 +97,7 @@
     <t>content-hub</t>
   </si>
   <si>
-    <t>2026-03-30T19:05:31.857Z</t>
+    <t>2026-03-30T19:07:05.352Z</t>
   </si>
   <si>
     <t>Ancestry Academy | Ancestry</t>
@@ -118,7 +118,7 @@
     <t>learning-directory</t>
   </si>
   <si>
-    <t>2026-03-30T18:25:09.146Z</t>
+    <t>2026-03-30T19:06:43.639Z</t>
   </si>
   <si>
     <t>AncestryDNA Learning Hub</t>

</xml_diff>